<commit_message>
updating helix effect finder
</commit_message>
<xml_diff>
--- a/hmwebsite/helix/data/models v3.50.xlsx
+++ b/hmwebsite/helix/data/models v3.50.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Dropbox\Html Tools\hmwebsite\hmwebsite\helix\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\hmon.ir\hmwebsite\helix\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{825810CF-80D0-426F-896C-8529571AFB87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCF62679-DDCE-49B8-8299-16FC783735AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3539" uniqueCount="1356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3539" uniqueCount="1357">
   <si>
     <t>Version</t>
   </si>
@@ -4103,6 +4103,9 @@
   </si>
   <si>
     <t>CAB_HX_2x12_Match_G25_NEW</t>
+  </si>
+  <si>
+    <t>Distortion,Noise Gate,Dynamics</t>
   </si>
 </sst>
 </file>
@@ -6029,7 +6032,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="12">
         <v>1</v>
       </c>
@@ -6058,7 +6061,7 @@
       </c>
       <c r="K47" s="13"/>
     </row>
-    <row r="48" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="12">
         <v>1</v>
       </c>
@@ -6089,7 +6092,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="12">
         <v>1</v>
       </c>
@@ -6122,7 +6125,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="12">
         <v>1</v>
       </c>
@@ -6151,7 +6154,7 @@
       </c>
       <c r="K50" s="13"/>
     </row>
-    <row r="51" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="12">
         <v>1</v>
       </c>
@@ -6182,7 +6185,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="12">
         <v>1</v>
       </c>
@@ -6213,7 +6216,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="12">
         <v>1</v>
       </c>
@@ -6244,7 +6247,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="54" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="12">
         <v>1</v>
       </c>
@@ -6275,7 +6278,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="55" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="12">
         <v>1</v>
       </c>
@@ -6308,7 +6311,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="56" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="12">
         <v>1</v>
       </c>
@@ -6339,7 +6342,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="57" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="12">
         <v>1</v>
       </c>
@@ -6370,7 +6373,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="58" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="12">
         <v>1</v>
       </c>
@@ -6401,7 +6404,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="59" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="12">
         <v>1</v>
       </c>
@@ -6432,7 +6435,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="60" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="12">
         <v>1</v>
       </c>
@@ -6463,7 +6466,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="12">
         <v>1</v>
       </c>
@@ -6494,7 +6497,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="62" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="12">
         <v>1</v>
       </c>
@@ -6525,7 +6528,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="63" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="12">
         <v>1</v>
       </c>
@@ -6556,7 +6559,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="64" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="12">
         <v>1</v>
       </c>
@@ -6587,7 +6590,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="65" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="12">
         <v>1</v>
       </c>
@@ -6618,7 +6621,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="66" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="12">
         <v>1</v>
       </c>
@@ -6649,7 +6652,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="67" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="12">
         <v>1</v>
       </c>
@@ -6680,7 +6683,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="68" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="12">
         <v>1</v>
       </c>
@@ -6711,7 +6714,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="69" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="12">
         <v>1</v>
       </c>
@@ -6742,7 +6745,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="70" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="12">
         <v>1</v>
       </c>
@@ -6773,7 +6776,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="71" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="12">
         <v>1</v>
       </c>
@@ -6804,7 +6807,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="72" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="12">
         <v>1</v>
       </c>
@@ -6835,7 +6838,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="73" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="12">
         <v>1</v>
       </c>
@@ -6866,7 +6869,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="74" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="12">
         <v>1</v>
       </c>
@@ -6897,7 +6900,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="75" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="12">
         <v>1</v>
       </c>
@@ -6928,7 +6931,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="76" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="12">
         <v>1</v>
       </c>
@@ -6959,7 +6962,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="77" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="12">
         <v>1</v>
       </c>
@@ -6988,7 +6991,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="78" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="12">
         <v>1</v>
       </c>
@@ -7019,7 +7022,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="79" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="12">
         <v>1</v>
       </c>
@@ -7050,7 +7053,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="80" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="12">
         <v>1</v>
       </c>
@@ -7081,7 +7084,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="81" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="12">
         <v>1</v>
       </c>
@@ -7110,7 +7113,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="82" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="12">
         <v>1</v>
       </c>
@@ -7141,7 +7144,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="83" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="12">
         <v>1</v>
       </c>
@@ -7170,7 +7173,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="84" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="12">
         <v>1</v>
       </c>
@@ -7201,7 +7204,7 @@
         <v>839</v>
       </c>
     </row>
-    <row r="85" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="12">
         <v>1</v>
       </c>
@@ -7230,7 +7233,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="86" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="12">
         <v>1</v>
       </c>
@@ -7259,7 +7262,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="87" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="12">
         <v>1</v>
       </c>
@@ -7290,7 +7293,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="88" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="12">
         <v>1</v>
       </c>
@@ -7319,7 +7322,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="89" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="12">
         <v>1</v>
       </c>
@@ -7348,7 +7351,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="90" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="12">
         <v>1</v>
       </c>
@@ -7379,7 +7382,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="91" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="12">
         <v>1</v>
       </c>
@@ -7408,7 +7411,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="92" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="12">
         <v>1</v>
       </c>
@@ -11389,7 +11392,7 @@
       </c>
       <c r="K230" s="16"/>
     </row>
-    <row r="231" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A231" s="15">
         <v>2.2000000000000002</v>
       </c>
@@ -11418,7 +11421,7 @@
       </c>
       <c r="K231" s="16"/>
     </row>
-    <row r="232" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A232" s="15">
         <v>2.2000000000000002</v>
       </c>
@@ -11449,7 +11452,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="233" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A233" s="15">
         <v>2.2000000000000002</v>
       </c>
@@ -11480,7 +11483,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="234" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A234" s="15">
         <v>2.2000000000000002</v>
       </c>
@@ -11509,7 +11512,7 @@
       </c>
       <c r="K234" s="16"/>
     </row>
-    <row r="235" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A235" s="15">
         <v>2.2000000000000002</v>
       </c>
@@ -11538,7 +11541,7 @@
       </c>
       <c r="K235" s="16"/>
     </row>
-    <row r="236" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A236" s="15">
         <v>2.2000000000000002</v>
       </c>
@@ -11569,7 +11572,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="237" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:11" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A237" s="15">
         <v>2.2000000000000002</v>
       </c>
@@ -15531,7 +15534,7 @@
         <v>860</v>
       </c>
     </row>
-    <row r="369" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A369" s="2">
         <v>2.9</v>
       </c>
@@ -15562,7 +15565,7 @@
         <v>947</v>
       </c>
     </row>
-    <row r="370" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A370" s="2">
         <v>2.9</v>
       </c>
@@ -15860,7 +15863,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="380" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A380" s="17">
         <v>3</v>
       </c>
@@ -15893,7 +15896,7 @@
         <v>990</v>
       </c>
     </row>
-    <row r="381" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A381" s="17">
         <v>3</v>
       </c>
@@ -15924,7 +15927,7 @@
         <v>1025</v>
       </c>
     </row>
-    <row r="382" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A382" s="17">
         <v>3</v>
       </c>
@@ -15949,7 +15952,7 @@
         <v>1008</v>
       </c>
       <c r="J382" s="18" t="s">
-        <v>12</v>
+        <v>1356</v>
       </c>
       <c r="K382" s="19" t="s">
         <v>1026</v>
@@ -16067,7 +16070,7 @@
         <v>1010</v>
       </c>
     </row>
-    <row r="387" spans="1:11" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A387" s="17">
         <v>3</v>
       </c>
@@ -17365,7 +17368,7 @@
         <v>1135</v>
       </c>
     </row>
-    <row r="433" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="433" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A433" s="51">
         <v>3.5</v>
       </c>
@@ -17396,7 +17399,7 @@
         <v>1291</v>
       </c>
     </row>
-    <row r="434" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="434" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A434" s="51">
         <v>3.5</v>
       </c>
@@ -17427,7 +17430,7 @@
         <v>1164</v>
       </c>
     </row>
-    <row r="435" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="435" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A435" s="51">
         <v>3.5</v>
       </c>
@@ -17458,7 +17461,7 @@
         <v>1165</v>
       </c>
     </row>
-    <row r="436" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="436" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A436" s="51">
         <v>3.5</v>
       </c>
@@ -17489,7 +17492,7 @@
         <v>1166</v>
       </c>
     </row>
-    <row r="437" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="437" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A437" s="51">
         <v>3.5</v>
       </c>
@@ -17520,7 +17523,7 @@
         <v>1167</v>
       </c>
     </row>
-    <row r="438" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="438" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A438" s="51">
         <v>3.5</v>
       </c>
@@ -17551,7 +17554,7 @@
         <v>1168</v>
       </c>
     </row>
-    <row r="439" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="439" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A439" s="51">
         <v>3.5</v>
       </c>
@@ -17582,7 +17585,7 @@
         <v>1169</v>
       </c>
     </row>
-    <row r="440" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="440" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A440" s="51">
         <v>3.5</v>
       </c>
@@ -17613,7 +17616,7 @@
         <v>1170</v>
       </c>
     </row>
-    <row r="441" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="441" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A441" s="51">
         <v>3.5</v>
       </c>
@@ -17644,7 +17647,7 @@
         <v>1171</v>
       </c>
     </row>
-    <row r="442" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="442" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A442" s="51">
         <v>3.5</v>
       </c>
@@ -17675,7 +17678,7 @@
         <v>1172</v>
       </c>
     </row>
-    <row r="443" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="443" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A443" s="51">
         <v>3.5</v>
       </c>
@@ -17706,7 +17709,7 @@
         <v>1173</v>
       </c>
     </row>
-    <row r="444" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="444" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A444" s="51">
         <v>3.5</v>
       </c>
@@ -17737,7 +17740,7 @@
         <v>1174</v>
       </c>
     </row>
-    <row r="445" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="445" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A445" s="51">
         <v>3.5</v>
       </c>
@@ -17768,7 +17771,7 @@
         <v>1175</v>
       </c>
     </row>
-    <row r="446" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="446" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A446" s="51">
         <v>3.5</v>
       </c>
@@ -17799,7 +17802,7 @@
         <v>1176</v>
       </c>
     </row>
-    <row r="447" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="447" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A447" s="51">
         <v>3.5</v>
       </c>
@@ -17830,7 +17833,7 @@
         <v>1177</v>
       </c>
     </row>
-    <row r="448" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="448" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A448" s="51">
         <v>3.5</v>
       </c>
@@ -17861,7 +17864,7 @@
         <v>1178</v>
       </c>
     </row>
-    <row r="449" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="449" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A449" s="51">
         <v>3.5</v>
       </c>
@@ -17892,7 +17895,7 @@
         <v>1179</v>
       </c>
     </row>
-    <row r="450" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="450" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A450" s="51">
         <v>3.5</v>
       </c>
@@ -17923,7 +17926,7 @@
         <v>1180</v>
       </c>
     </row>
-    <row r="451" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="451" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A451" s="51">
         <v>3.5</v>
       </c>
@@ -17954,7 +17957,7 @@
         <v>1181</v>
       </c>
     </row>
-    <row r="452" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="452" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A452" s="51">
         <v>3.5</v>
       </c>
@@ -17985,7 +17988,7 @@
         <v>1182</v>
       </c>
     </row>
-    <row r="453" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="453" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A453" s="51">
         <v>3.5</v>
       </c>
@@ -18016,7 +18019,7 @@
         <v>1206</v>
       </c>
     </row>
-    <row r="454" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="454" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A454" s="51">
         <v>3.5</v>
       </c>
@@ -18047,7 +18050,7 @@
         <v>1207</v>
       </c>
     </row>
-    <row r="455" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="455" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A455" s="51">
         <v>3.5</v>
       </c>
@@ -18078,7 +18081,7 @@
         <v>1205</v>
       </c>
     </row>
-    <row r="456" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="456" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A456" s="51">
         <v>3.5</v>
       </c>
@@ -18451,7 +18454,7 @@
         <v>1227</v>
       </c>
     </row>
-    <row r="469" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="469" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A469" s="51">
         <v>3.5</v>
       </c>
@@ -18480,7 +18483,7 @@
         <v>1268</v>
       </c>
     </row>
-    <row r="470" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="470" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A470" s="51">
         <v>3.5</v>
       </c>
@@ -18509,7 +18512,7 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="471" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="471" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A471" s="51">
         <v>3.5</v>
       </c>
@@ -18538,7 +18541,7 @@
         <v>1278</v>
       </c>
     </row>
-    <row r="472" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="472" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A472" s="51">
         <v>3.5</v>
       </c>
@@ -18567,7 +18570,7 @@
         <v>1273</v>
       </c>
     </row>
-    <row r="473" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="473" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A473" s="51">
         <v>3.5</v>
       </c>
@@ -18681,7 +18684,7 @@
         <v>1319</v>
       </c>
     </row>
-    <row r="477" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="477" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A477" s="44">
         <v>3.6</v>
       </c>
@@ -18710,7 +18713,7 @@
         <v>1303</v>
       </c>
     </row>
-    <row r="478" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="478" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A478" s="44">
         <v>3.6</v>
       </c>
@@ -18739,7 +18742,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="479" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="479" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A479" s="44">
         <v>3.6</v>
       </c>
@@ -18768,7 +18771,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="480" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="480" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A480" s="44">
         <v>3.6</v>
       </c>
@@ -18799,7 +18802,7 @@
         <v>1306</v>
       </c>
     </row>
-    <row r="481" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="481" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A481" s="44">
         <v>3.6</v>
       </c>
@@ -18830,7 +18833,7 @@
         <v>1307</v>
       </c>
     </row>
-    <row r="482" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="482" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A482" s="44">
         <v>3.6</v>
       </c>
@@ -18861,7 +18864,7 @@
         <v>1308</v>
       </c>
     </row>
-    <row r="483" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="483" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A483" s="44">
         <v>3.6</v>
       </c>
@@ -18890,7 +18893,7 @@
         <v>1309</v>
       </c>
     </row>
-    <row r="484" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="484" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A484" s="44">
         <v>3.6</v>
       </c>
@@ -18917,7 +18920,7 @@
         <v>1310</v>
       </c>
     </row>
-    <row r="485" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="485" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A485" s="44">
         <v>3.6</v>
       </c>
@@ -19004,7 +19007,7 @@
         <v>1315</v>
       </c>
     </row>
-    <row r="488" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="488" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A488" s="57">
         <v>3.6</v>
       </c>
@@ -19033,7 +19036,7 @@
         <v>1335</v>
       </c>
     </row>
-    <row r="489" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="489" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A489" s="44">
         <v>3.6</v>
       </c>
@@ -19064,9 +19067,10 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:K489" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="1">
+    <filterColumn colId="3">
       <filters>
-        <filter val="Cab"/>
+        <filter val="Horizon Drive"/>
+        <filter val="Horizon Gate"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>